<commit_message>
add part word3 excel
</commit_message>
<xml_diff>
--- a/WORD/2_22_12.xlsx
+++ b/WORD/2_22_12.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\N2_2025_12\WORD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DC15576-25BF-461E-96C6-56FA3ED37E77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2FB637C-FFFA-4212-8CE7-09B4E30470CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14820" yWindow="4275" windowWidth="23580" windowHeight="9255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8505" yWindow="1605" windowWidth="23580" windowHeight="17835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="221">
   <si>
     <t>Fre</t>
   </si>
@@ -444,88 +444,301 @@
     <t>求職</t>
   </si>
   <si>
+    <t>情</t>
+  </si>
+  <si>
+    <t>じょう</t>
+  </si>
+  <si>
+    <t>情，感情</t>
+  </si>
+  <si>
+    <t>職業</t>
+  </si>
+  <si>
+    <t>しょくぎょう</t>
+  </si>
+  <si>
+    <t>职业</t>
+  </si>
+  <si>
+    <t>俳優</t>
+  </si>
+  <si>
+    <t>はいゆう</t>
+  </si>
+  <si>
+    <t>演员</t>
+  </si>
+  <si>
+    <t>男優</t>
+  </si>
+  <si>
+    <t>だんゆう</t>
+  </si>
+  <si>
+    <t>女優</t>
+  </si>
+  <si>
+    <t>じょゆう</t>
+  </si>
+  <si>
+    <t>声優</t>
+  </si>
+  <si>
+    <t>せいゆう</t>
+  </si>
+  <si>
+    <t>逃れる</t>
+  </si>
+  <si>
+    <t>のがれる</t>
+  </si>
+  <si>
+    <t>逃避；避开；摆脱</t>
+  </si>
+  <si>
+    <t>別れる</t>
+  </si>
+  <si>
+    <t>わかれる</t>
+  </si>
+  <si>
+    <t>离别，分手</t>
+  </si>
+  <si>
+    <t>離れる</t>
+  </si>
+  <si>
+    <t>はなれる</t>
+  </si>
+  <si>
+    <t>离开;分离;相隔;脱离</t>
+  </si>
+  <si>
+    <t>備える</t>
+  </si>
+  <si>
+    <t>そなえる</t>
+  </si>
+  <si>
+    <t>准备；防备</t>
+  </si>
+  <si>
+    <t>自信</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>じしん</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>技術</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ぎじゅつ</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>経験</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>けいけん</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>经验；经历</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>きゅうしょく</t>
-  </si>
-  <si>
-    <t>情</t>
-  </si>
-  <si>
-    <t>じょう</t>
-  </si>
-  <si>
-    <t>情，感情</t>
-  </si>
-  <si>
-    <t>職業</t>
-  </si>
-  <si>
-    <t>しょくぎょう</t>
-  </si>
-  <si>
-    <t>职业</t>
-  </si>
-  <si>
-    <t>俳優</t>
-  </si>
-  <si>
-    <t>はいゆう</t>
-  </si>
-  <si>
-    <t>演员</t>
-  </si>
-  <si>
-    <t>男優</t>
-  </si>
-  <si>
-    <t>だんゆう</t>
-  </si>
-  <si>
-    <t>女優</t>
-  </si>
-  <si>
-    <t>じょゆう</t>
-  </si>
-  <si>
-    <t>声優</t>
-  </si>
-  <si>
-    <t>せいゆう</t>
-  </si>
-  <si>
-    <t>逃れる</t>
-  </si>
-  <si>
-    <t>のがれる</t>
-  </si>
-  <si>
-    <t>逃避；避开；摆脱</t>
-  </si>
-  <si>
-    <t>別れる</t>
-  </si>
-  <si>
-    <t>わかれる</t>
-  </si>
-  <si>
-    <t>离别，分手</t>
-  </si>
-  <si>
-    <t>離れる</t>
-  </si>
-  <si>
-    <t>はなれる</t>
-  </si>
-  <si>
-    <t>离开;分离;相隔;脱离</t>
-  </si>
-  <si>
-    <t>備える</t>
-  </si>
-  <si>
-    <t>そなえる</t>
-  </si>
-  <si>
-    <t>准备；防备</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>体力</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>たいりょく</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>新聞</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>しんぶん</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>报纸</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>一転する</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>いってんする</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>突然改变</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>すっかり</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>完全；彻底；全部</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>やっと</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>终于；好不容易</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>先</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>さき</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>前面；尖端</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>尖る</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>とがる</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>变尖；紧张；敏感；发怒</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>太い</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ふとい</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>粗；胖；厚</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>くだらない</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>无价值的;无聊的</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>頑固</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>がんこ</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>(性格)顽固</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ふた</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>(瓶子)盖子</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>打ち合わせ</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>うちあわせ</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>事前协商；讨论会</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ないか</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>是否…</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>中断</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ちゅうだん</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>暂停；中止；间断</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>断る</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ことわる</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>拒绝；谢绝；事先通知；事先说好</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>やむ</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>停止；中止；结束</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ベテラン</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>老手；经验丰富的人；资深者</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>荒れる</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>あれる</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>（天气）恶劣；（海面）波涛汹涌；（皮肤）粗糙</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -896,7 +1109,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E89"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -1617,7 +1830,7 @@
         <v>139</v>
       </c>
       <c r="D58" t="s">
-        <v>140</v>
+        <v>174</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.15">
@@ -1625,13 +1838,13 @@
         <v>0</v>
       </c>
       <c r="B59" t="s">
+        <v>140</v>
+      </c>
+      <c r="D59" t="s">
         <v>141</v>
       </c>
-      <c r="D59" t="s">
+      <c r="E59" t="s">
         <v>142</v>
-      </c>
-      <c r="E59" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.15">
@@ -1639,13 +1852,13 @@
         <v>1</v>
       </c>
       <c r="B60" t="s">
+        <v>143</v>
+      </c>
+      <c r="D60" t="s">
         <v>144</v>
       </c>
-      <c r="D60" t="s">
+      <c r="E60" t="s">
         <v>145</v>
-      </c>
-      <c r="E60" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.15">
@@ -1653,13 +1866,13 @@
         <v>1</v>
       </c>
       <c r="B61" t="s">
+        <v>146</v>
+      </c>
+      <c r="D61" t="s">
         <v>147</v>
       </c>
-      <c r="D61" t="s">
+      <c r="E61" t="s">
         <v>148</v>
-      </c>
-      <c r="E61" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.15">
@@ -1667,10 +1880,10 @@
         <v>0</v>
       </c>
       <c r="B62" t="s">
+        <v>149</v>
+      </c>
+      <c r="D62" t="s">
         <v>150</v>
-      </c>
-      <c r="D62" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.15">
@@ -1678,10 +1891,10 @@
         <v>0</v>
       </c>
       <c r="B63" t="s">
+        <v>151</v>
+      </c>
+      <c r="D63" t="s">
         <v>152</v>
-      </c>
-      <c r="D63" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.15">
@@ -1689,10 +1902,10 @@
         <v>0</v>
       </c>
       <c r="B64" t="s">
+        <v>153</v>
+      </c>
+      <c r="D64" t="s">
         <v>154</v>
-      </c>
-      <c r="D64" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.15">
@@ -1700,13 +1913,13 @@
         <v>0</v>
       </c>
       <c r="B65" t="s">
+        <v>155</v>
+      </c>
+      <c r="D65" t="s">
         <v>156</v>
       </c>
-      <c r="D65" t="s">
+      <c r="E65" t="s">
         <v>157</v>
-      </c>
-      <c r="E65" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.15">
@@ -1714,13 +1927,13 @@
         <v>1</v>
       </c>
       <c r="B66" t="s">
+        <v>158</v>
+      </c>
+      <c r="D66" t="s">
         <v>159</v>
       </c>
-      <c r="D66" t="s">
+      <c r="E66" t="s">
         <v>160</v>
-      </c>
-      <c r="E66" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.15">
@@ -1728,13 +1941,13 @@
         <v>0</v>
       </c>
       <c r="B67" t="s">
+        <v>161</v>
+      </c>
+      <c r="D67" t="s">
         <v>162</v>
       </c>
-      <c r="D67" t="s">
+      <c r="E67" t="s">
         <v>163</v>
-      </c>
-      <c r="E67" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.15">
@@ -1742,13 +1955,277 @@
         <v>0</v>
       </c>
       <c r="B68" t="s">
+        <v>164</v>
+      </c>
+      <c r="D68" t="s">
         <v>165</v>
       </c>
-      <c r="D68" t="s">
+      <c r="E68" t="s">
         <v>166</v>
       </c>
-      <c r="E68" t="s">
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A69">
+        <v>0</v>
+      </c>
+      <c r="B69" t="s">
         <v>167</v>
+      </c>
+      <c r="D69" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A70">
+        <v>0</v>
+      </c>
+      <c r="B70" t="s">
+        <v>169</v>
+      </c>
+      <c r="D70" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A71">
+        <v>0</v>
+      </c>
+      <c r="B71" t="s">
+        <v>171</v>
+      </c>
+      <c r="D71" t="s">
+        <v>172</v>
+      </c>
+      <c r="E71" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A72">
+        <v>0</v>
+      </c>
+      <c r="B72" t="s">
+        <v>175</v>
+      </c>
+      <c r="D72" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A73">
+        <v>0</v>
+      </c>
+      <c r="B73" t="s">
+        <v>177</v>
+      </c>
+      <c r="D73" t="s">
+        <v>178</v>
+      </c>
+      <c r="E73" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A74">
+        <v>0</v>
+      </c>
+      <c r="B74" t="s">
+        <v>180</v>
+      </c>
+      <c r="D74" t="s">
+        <v>181</v>
+      </c>
+      <c r="E74" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A75">
+        <v>0</v>
+      </c>
+      <c r="B75" t="s">
+        <v>183</v>
+      </c>
+      <c r="D75" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A76">
+        <v>0</v>
+      </c>
+      <c r="B76" t="s">
+        <v>185</v>
+      </c>
+      <c r="D76" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A77">
+        <v>0</v>
+      </c>
+      <c r="B77" t="s">
+        <v>187</v>
+      </c>
+      <c r="D77" t="s">
+        <v>188</v>
+      </c>
+      <c r="E77" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A78">
+        <v>0</v>
+      </c>
+      <c r="B78" t="s">
+        <v>190</v>
+      </c>
+      <c r="D78" t="s">
+        <v>191</v>
+      </c>
+      <c r="E78" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A79">
+        <v>0</v>
+      </c>
+      <c r="B79" t="s">
+        <v>193</v>
+      </c>
+      <c r="D79" t="s">
+        <v>194</v>
+      </c>
+      <c r="E79" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A80">
+        <v>0</v>
+      </c>
+      <c r="B80" t="s">
+        <v>196</v>
+      </c>
+      <c r="E80" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A81">
+        <v>0</v>
+      </c>
+      <c r="B81" t="s">
+        <v>198</v>
+      </c>
+      <c r="D81" t="s">
+        <v>199</v>
+      </c>
+      <c r="E81" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A82">
+        <v>0</v>
+      </c>
+      <c r="B82" t="s">
+        <v>201</v>
+      </c>
+      <c r="E82" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A83">
+        <v>0</v>
+      </c>
+      <c r="B83" t="s">
+        <v>203</v>
+      </c>
+      <c r="D83" t="s">
+        <v>204</v>
+      </c>
+      <c r="E83" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A84">
+        <v>0</v>
+      </c>
+      <c r="B84" t="s">
+        <v>206</v>
+      </c>
+      <c r="D84" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A85">
+        <v>0</v>
+      </c>
+      <c r="B85" t="s">
+        <v>208</v>
+      </c>
+      <c r="D85" t="s">
+        <v>209</v>
+      </c>
+      <c r="E85" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A86">
+        <v>0</v>
+      </c>
+      <c r="B86" t="s">
+        <v>211</v>
+      </c>
+      <c r="D86" t="s">
+        <v>212</v>
+      </c>
+      <c r="E86" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A87">
+        <v>0</v>
+      </c>
+      <c r="B87" t="s">
+        <v>214</v>
+      </c>
+      <c r="E87" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A88">
+        <v>0</v>
+      </c>
+      <c r="B88" t="s">
+        <v>216</v>
+      </c>
+      <c r="E88" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A89">
+        <v>0</v>
+      </c>
+      <c r="B89" t="s">
+        <v>218</v>
+      </c>
+      <c r="D89" t="s">
+        <v>219</v>
+      </c>
+      <c r="E89" t="s">
+        <v>220</v>
       </c>
     </row>
   </sheetData>

</xml_diff>